<commit_message>
update： 1.ecFSEOF. 2.evaluation method
</commit_message>
<xml_diff>
--- a/data/experiment_targets/detailed_collect/ffa_exp_data.xlsx
+++ b/data/experiment_targets/detailed_collect/ffa_exp_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\github\strainOptimizer\data\experiment_targets\detailed_collect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577BF087-F94C-4A73-B1D2-6C1BC3207A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{627ADF3E-79C6-4124-A6A8-B491D5E4729E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27495" yWindow="8370" windowWidth="16410" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29325" yWindow="6960" windowWidth="15930" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="70">
   <si>
     <t>geneID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -268,6 +268,23 @@
   </si>
   <si>
     <t>10.1038/ncomms11711</t>
+  </si>
+  <si>
+    <t>OE</t>
+  </si>
+  <si>
+    <t>KD</t>
+  </si>
+  <si>
+    <t>KO</t>
+  </si>
+  <si>
+    <t>OE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KO</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -598,6 +615,8 @@
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="21.75" customWidth="1"/>
+    <col min="3" max="3" width="22.875" customWidth="1"/>
     <col min="6" max="6" width="30.25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -632,7 +651,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -652,7 +671,7 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -672,7 +691,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -692,7 +711,7 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -712,7 +731,7 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -732,7 +751,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -752,7 +771,7 @@
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>66</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -772,7 +791,7 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -792,7 +811,7 @@
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -812,7 +831,7 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -832,7 +851,7 @@
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -852,7 +871,7 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -872,7 +891,7 @@
         <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -892,7 +911,7 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -912,7 +931,7 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -932,7 +951,7 @@
         <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -949,7 +968,7 @@
         <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -966,7 +985,7 @@
         <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D19">
         <v>1</v>

</xml_diff>